<commit_message>
v5: players, lineup, reset button, help dialog, sheet with players/lineups tabs
</commit_message>
<xml_diff>
--- a/Boule-matcher-mall.xlsx
+++ b/Boule-matcher-mall.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="68">
   <si>
     <t xml:space="preserve">Boule Score Tracker</t>
   </si>
@@ -120,10 +120,14 @@
   <si>
     <t xml:space="preserve">/**
  * Boule Score Tracker — Google Sheets webhook
- * Tar emot POST-JSON från Boule-appen och sparar en rad per match.
+ * Tar emot POST-JSON från Boule-appen.
+ * Skriver till tre flikar: Matcher, Lagsättningar, Spelare.
  */
-const SHEET_NAME = 'Matcher';
-const HEADERS = [
+const MATCH_SHEET = 'Matcher';
+const LINEUP_SHEET = 'Lagsättningar';
+const PLAYERS_SHEET = 'Spelare';
+const MATCH_HEADERS = [
+  'Match-ID',
   'Sparad',
   'Startade',
   'Slutade',
@@ -134,39 +138,28 @@
   'GPS-noggrannhet (m)',
   'Mål',
   'Lag 1',
+  'Spelare Lag 1',
   'Poäng 1',
   'Lag 2',
+  'Spelare Lag 2',
   'Poäng 2',
   'Vinnare',
   'Antal omgångar',
   'Omgångar (JSON)',
 ];
+const LINEUP_HEADERS = ['Match-ID', 'Sparad', 'Lag', 'Lagnamn', 'Spelare'];
+const PLAYER_HEADERS = ['Spelare', 'Matcher', 'Vinster', 'Senast sedd'];
 function doPost(e) {
   try {
     const raw = e &amp;&amp; e.postData &amp;&amp; e.postData.contents;
     if (!raw) throw new Error('Tom request body');
     const data = JSON.parse(raw);
-    const sheet = getOrCreateSheet_();
-    const row = [
-      data.savedAt || new Date().toISOString(),
-      data.startedAt || '',
-      data.endedAt || '',
-      data.timezone || '',
-      data.place || '',
-      data.location ? data.location.lat : '',
-      data.location ? data.location.lng : '',
-      data.location ? data.location.accuracy : '',
-      data.target || '',
-      (data.teams &amp;&amp; data.teams[0] &amp;&amp; data.teams[0].name) || '',
-      (data.teams &amp;&amp; data.teams[0] &amp;&amp; data.teams[0].score) || 0,
-      (data.teams &amp;&amp; data.teams[1] &amp;&amp; data.teams[1].name) || '',
-      (data.teams &amp;&amp; data.teams[1] &amp;&amp; data.teams[1].score) || 0,
-      data.winner || '',
-      (data.rounds &amp;&amp; data.rounds.length) || 0,
-      JSON.stringify(data.rounds || []),
-    ];
-    sheet.appendRow(row);
-    return json_({ ok: true, row: sheet.getLastRow() });
+    const matchId = (data.endedAt || data.savedAt || new Date().toISOString()) + '-' +
+      Math.random().toString(36).slice(2, 7);
+    writeMatch_(matchId, data);
+    writeLineups_(matchId, data);
+    upsertPlayers_(data);
+    return json_({ ok: true, matchId: matchId });
   } catch (err) {
     return json_({ ok: false, error: String(err) });
   }
@@ -174,17 +167,82 @@
 function doGet() {
   return json_({
     ok: true,
-    service: 'Boule webhook',
+    service: 'Boule webhook v2',
     usage: 'POST JSON från Boule-appen till denna URL',
   });
 }
-function getOrCreateSheet_() {
+function writeMatch_(matchId, data) {
+  const sheet = getOrCreateSheet_(MATCH_SHEET, MATCH_HEADERS);
+  const t1 = (data.teams &amp;&amp; data.teams[0]) || {};
+  const t2 = (data.teams &amp;&amp; data.teams[1]) || {};
+  sheet.appendRow([
+    matchId,
+    data.savedAt || new Date().toISOString(),
+    data.startedAt || '',
+    data.endedAt || '',
+    data.timezone || '',
+    data.place || '',
+    data.location ? data.location.lat : '',
+    data.location ? data.location.lng : '',
+    data.location ? data.location.accuracy : '',
+    data.target || '',
+    t1.name || '',
+    (t1.players || []).join(', '),
+    t1.score || 0,
+    t2.name || '',
+    (t2.players || []).join(', '),
+    t2.score || 0,
+    data.winner || '',
+    (data.rounds &amp;&amp; data.rounds.length) || 0,
+    JSON.stringify(data.rounds || []),
+  ]);
+}
+function writeLineups_(matchId, data) {
+  const sheet = getOrCreateSheet_(LINEUP_SHEET, LINEUP_HEADERS);
+  const saved = data.savedAt || new Date().toISOString();
+  (data.teams || []).forEach((team, idx) =&gt; {
+    (team.players || []).forEach((p) =&gt; {
+      sheet.appendRow([matchId, saved, 'Lag ' + (idx + 1), team.name || '', p]);
+    });
+  });
+}
+function upsertPlayers_(data) {
+  const sheet = getOrCreateSheet_(PLAYERS_SHEET, PLAYER_HEADERS);
+  const values = sheet.getDataRange().getValues(); // inkl header
+  const indexByName = {};
+  for (let r = 1; r &lt; values.length; r++) {
+    indexByName[String(values[r][0]).toLowerCase()] = r + 1; // 1-indexerat radnummer
+  }
+  const saved = data.savedAt || new Date().toISOString();
+  const allPlayers = [];
+  (data.teams || []).forEach((team) =&gt; {
+    (team.players || []).forEach((p) =&gt; {
+      allPlayers.push({ name: p, team: team.name });
+    });
+  });
+  const winner = data.winner;
+  allPlayers.forEach((pl) =&gt; {
+    const key = pl.name.toLowerCase();
+    const existingRow = indexByName[key];
+    if (existingRow) {
+      const matches = Number(sheet.getRange(existingRow, 2).getValue()) || 0;
+      const wins = Number(sheet.getRange(existingRow, 3).getValue()) || 0;
+      sheet.getRange(existingRow, 2).setValue(matches + 1);
+      if (pl.team === winner) sheet.getRange(existingRow, 3).setValue(wins + 1);
+      sheet.getRange(existingRow, 4).setValue(saved);
+    } else {
+      sheet.appendRow([pl.name, 1, pl.team === winner ? 1 : 0, saved]);
+      indexByName[key] = sheet.getLastRow();
+    }
+  });
+}
+function getOrCreateSheet_(name, headers) {
   const ss = SpreadsheetApp.getActiveSpreadsheet();
-  let sheet = ss.getSheetByName(SHEET_NAME);
-  if (!sheet) sheet = ss.insertSheet(SHEET_NAME);
+  let sheet = ss.getSheetByName(name);
+  if (!sheet) sheet = ss.insertSheet(name);
   if (sheet.getLastRow() === 0) {
-    sheet.appendRow(HEADERS);
-    sheet.getRange(1, 1, 1, HEADERS.length).setFontWeight('bold');
+    sheet.appendRow(headers);
+    sheet.getRange(1, 1, 1, headers.length).setFontWeight('bold');
     sheet.setFrozenRows(1);
   }
   return sheet;
@@ -197,6 +255,9 @@
 </t>
   </si>
   <si>
+    <t xml:space="preserve">Match-ID</t>
+  </si>
+  <si>
     <t xml:space="preserve">Sparad</t>
   </si>
   <si>
@@ -227,12 +288,18 @@
     <t xml:space="preserve">Lag 1</t>
   </si>
   <si>
+    <t xml:space="preserve">Spelare Lag 1</t>
+  </si>
+  <si>
     <t xml:space="preserve">Poäng 1</t>
   </si>
   <si>
     <t xml:space="preserve">Lag 2</t>
   </si>
   <si>
+    <t xml:space="preserve">Spelare Lag 2</t>
+  </si>
+  <si>
     <t xml:space="preserve">Poäng 2</t>
   </si>
   <si>
@@ -245,6 +312,9 @@
     <t xml:space="preserve">Omgångar (JSON)</t>
   </si>
   <si>
+    <t xml:space="preserve">2026-04-18T20:15:30.000Z-ab12c</t>
+  </si>
+  <si>
     <t xml:space="preserve">2026-04-18T20:15:30.000Z</t>
   </si>
   <si>
@@ -257,15 +327,21 @@
     <t xml:space="preserve">Europe/Stockholm</t>
   </si>
   <si>
-    <t xml:space="preserve">Sexdrega gräsmatta</t>
+    <t xml:space="preserve">Sexdrega, Svenljunga, Sverige</t>
   </si>
   <si>
     <t xml:space="preserve">Tjejerna</t>
   </si>
   <si>
+    <t xml:space="preserve">Anna, Mia</t>
+  </si>
+  <si>
     <t xml:space="preserve">Killarna</t>
   </si>
   <si>
+    <t xml:space="preserve">Erik, Johan</t>
+  </si>
+  <si>
     <t xml:space="preserve">[{"n":1,"team":"Tjejerna","points":2,"tally":[2,0]}, …]</t>
   </si>
   <si>
@@ -288,6 +364,9 @@
   </si>
   <si>
     <t xml:space="preserve">Snitt omgångar per match</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Antal unika spelare</t>
   </si>
   <si>
     <t xml:space="preserve">Per lag</t>
@@ -964,7 +1043,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="1209.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="2091.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="6" t="s">
         <v>20</v>
       </c>
@@ -985,22 +1064,25 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P4"/>
+  <dimension ref="A1:S4"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="1" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="50"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1052,60 +1134,78 @@
       <c r="P1" s="7" t="s">
         <v>36</v>
       </c>
+      <c r="Q1" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="R1" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="S1" s="7" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="F2" s="9" t="n">
+        <v>44</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="G2" s="9" t="n">
         <v>57.82015</v>
       </c>
-      <c r="G2" s="9" t="n">
+      <c r="H2" s="9" t="n">
         <v>13.19043</v>
       </c>
-      <c r="H2" s="10" t="n">
+      <c r="I2" s="10" t="n">
         <v>15</v>
       </c>
-      <c r="I2" s="10" t="n">
+      <c r="J2" s="10" t="n">
         <v>13</v>
       </c>
-      <c r="J2" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="K2" s="10" t="n">
+      <c r="K2" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="L2" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="M2" s="10" t="n">
         <v>13</v>
       </c>
-      <c r="L2" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="M2" s="10" t="n">
+      <c r="N2" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="O2" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="P2" s="10" t="n">
         <v>9</v>
       </c>
-      <c r="N2" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="O2" s="10" t="n">
+      <c r="Q2" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="R2" s="10" t="n">
         <v>11</v>
       </c>
-      <c r="P2" s="8" t="s">
-        <v>44</v>
+      <c r="S2" s="8" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="B4" s="11"/>
       <c r="C4" s="11"/>
@@ -1122,10 +1222,13 @@
       <c r="N4" s="11"/>
       <c r="O4" s="11"/>
       <c r="P4" s="11"/>
+      <c r="Q4" s="11"/>
+      <c r="R4" s="11"/>
+      <c r="S4" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A4:P4"/>
+    <mergeCell ref="A4:S4"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1153,239 +1256,248 @@
     <row r="1" customFormat="false" ht="9.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="2" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="2" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="9.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="12" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="C5" s="13" t="n">
-        <f aca="false">COUNTA(Matcher!N:N)-1</f>
+        <f aca="false">COUNTA(Matcher!Q:Q)-1</f>
         <v>1</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="12" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="C6" s="13" t="n">
-        <f aca="false">COUNTIF(Matcher!N:N,"Tjejerna")</f>
+        <f aca="false">COUNTIF(Matcher!Q:Q,"Tjejerna")</f>
         <v>1</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="12" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="C7" s="13" t="n">
-        <f aca="false">COUNTIF(Matcher!N:N,"Killarna")</f>
+        <f aca="false">COUNTIF(Matcher!Q:Q,"Killarna")</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="12" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="C8" s="14" t="n">
-        <f aca="false">IFERROR(AVERAGE(Matcher!O2:O1000),0)</f>
+        <f aca="false">IFERROR(AVERAGE(Matcher!R2:R1000),0)</f>
         <v>11</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B9" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="C9" s="13" t="n">
+        <f aca="false">IFERROR(COUNTA(spelare!a:a)-1,0)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="15" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="16" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="17" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="C12" s="18" t="n">
-        <f aca="false">COUNTIF(Matcher!N:N,B12)</f>
+        <f aca="false">COUNTIF(Matcher!Q:Q,B12)</f>
         <v>1</v>
       </c>
       <c r="D12" s="18" t="n">
-        <f aca="false">SUMIF(Matcher!J:J,B12,Matcher!K:K)+SUMIF(Matcher!L:L,B12,Matcher!M:M)</f>
+        <f aca="false">SUMIF(Matcher!K:K,B12,Matcher!M:M)+SUMIF(Matcher!N:N,B12,Matcher!P:P)</f>
         <v>13</v>
       </c>
       <c r="E12" s="19" t="str">
-        <f aca="false">IFERROR(maxifs(Matcher!C:C,Matcher!N:N,B12),"—")</f>
+        <f aca="false">IFERROR(maxifs(Matcher!D:D,Matcher!Q:Q,B12),"—")</f>
         <v>—</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="17" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="C13" s="18" t="n">
-        <f aca="false">COUNTIF(Matcher!N:N,B13)</f>
+        <f aca="false">COUNTIF(Matcher!Q:Q,B13)</f>
         <v>0</v>
       </c>
       <c r="D13" s="18" t="n">
-        <f aca="false">SUMIF(Matcher!J:J,B13,Matcher!K:K)+SUMIF(Matcher!L:L,B13,Matcher!M:M)</f>
+        <f aca="false">SUMIF(Matcher!K:K,B13,Matcher!M:M)+SUMIF(Matcher!N:N,B13,Matcher!P:P)</f>
         <v>9</v>
       </c>
       <c r="E13" s="19" t="str">
-        <f aca="false">IFERROR(maxifs(Matcher!C:C,Matcher!N:N,B13),"—")</f>
+        <f aca="false">IFERROR(maxifs(Matcher!D:D,Matcher!Q:Q,B13),"—")</f>
         <v>—</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B15" s="15" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="16" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="C16" s="16" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D16" s="16" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="E16" s="16" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F16" s="16" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B17" s="20" t="n">
-        <f aca="false">IFERROR(INDEX(Matcher!C:C,COUNTA(Matcher!A:A)-1-0+1),"—")</f>
-        <v>0</v>
-      </c>
-      <c r="C17" s="20" t="n">
-        <f aca="false">IFERROR(INDEX(Matcher!J:J,COUNTA(Matcher!A:A)-1-0+1),"—")</f>
-        <v>0</v>
+      <c r="B17" s="20" t="str">
+        <f aca="false">IFERROR(INDEX(Matcher!D:D,COUNTA(Matcher!B:B)-1-0+1),"—")</f>
+        <v>2026-04-18T20:15:28.000Z</v>
+      </c>
+      <c r="C17" s="20" t="str">
+        <f aca="false">IFERROR(INDEX(Matcher!K:K,COUNTA(Matcher!B:B)-1-0+1),"—")</f>
+        <v>Tjejerna</v>
       </c>
       <c r="D17" s="20" t="str">
-        <f aca="false">IFERROR(INDEX(Matcher!K:K,COUNTA(Matcher!A:A)-1-0+1)&amp;" – "&amp;INDEX(Matcher!M:M,COUNTA(Matcher!A:A)-1-0+1),"—")</f>
-        <v> – </v>
-      </c>
-      <c r="E17" s="20" t="n">
-        <f aca="false">IFERROR(INDEX(Matcher!L:L,COUNTA(Matcher!A:A)-1-0+1),"—")</f>
-        <v>0</v>
-      </c>
-      <c r="F17" s="20" t="n">
-        <f aca="false">IFERROR(INDEX(Matcher!N:N,COUNTA(Matcher!A:A)-1-0+1),"—")</f>
-        <v>0</v>
+        <f aca="false">IFERROR(INDEX(Matcher!M:M,COUNTA(Matcher!B:B)-1-0+1)&amp;" – "&amp;INDEX(Matcher!P:P,COUNTA(Matcher!B:B)-1-0+1),"—")</f>
+        <v>13 – 9</v>
+      </c>
+      <c r="E17" s="20" t="str">
+        <f aca="false">IFERROR(INDEX(Matcher!N:N,COUNTA(Matcher!B:B)-1-0+1),"—")</f>
+        <v>Killarna</v>
+      </c>
+      <c r="F17" s="20" t="str">
+        <f aca="false">IFERROR(INDEX(Matcher!Q:Q,COUNTA(Matcher!B:B)-1-0+1),"—")</f>
+        <v>Tjejerna</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="20" t="str">
-        <f aca="false">IFERROR(INDEX(Matcher!C:C,COUNTA(Matcher!A:A)-1-1+1),"—")</f>
-        <v>2026-04-18T20:15:28.000Z</v>
+        <f aca="false">IFERROR(INDEX(Matcher!D:D,COUNTA(Matcher!B:B)-1-1+1),"—")</f>
+        <v>Slutade</v>
       </c>
       <c r="C18" s="20" t="str">
-        <f aca="false">IFERROR(INDEX(Matcher!J:J,COUNTA(Matcher!A:A)-1-1+1),"—")</f>
-        <v>Tjejerna</v>
+        <f aca="false">IFERROR(INDEX(Matcher!K:K,COUNTA(Matcher!B:B)-1-1+1),"—")</f>
+        <v>Lag 1</v>
       </c>
       <c r="D18" s="20" t="str">
-        <f aca="false">IFERROR(INDEX(Matcher!K:K,COUNTA(Matcher!A:A)-1-1+1)&amp;" – "&amp;INDEX(Matcher!M:M,COUNTA(Matcher!A:A)-1-1+1),"—")</f>
-        <v>13 – 9</v>
+        <f aca="false">IFERROR(INDEX(Matcher!M:M,COUNTA(Matcher!B:B)-1-1+1)&amp;" – "&amp;INDEX(Matcher!P:P,COUNTA(Matcher!B:B)-1-1+1),"—")</f>
+        <v>Poäng 1 – Poäng 2</v>
       </c>
       <c r="E18" s="20" t="str">
-        <f aca="false">IFERROR(INDEX(Matcher!L:L,COUNTA(Matcher!A:A)-1-1+1),"—")</f>
-        <v>Killarna</v>
+        <f aca="false">IFERROR(INDEX(Matcher!N:N,COUNTA(Matcher!B:B)-1-1+1),"—")</f>
+        <v>Lag 2</v>
       </c>
       <c r="F18" s="20" t="str">
-        <f aca="false">IFERROR(INDEX(Matcher!N:N,COUNTA(Matcher!A:A)-1-1+1),"—")</f>
-        <v>Tjejerna</v>
+        <f aca="false">IFERROR(INDEX(Matcher!Q:Q,COUNTA(Matcher!B:B)-1-1+1),"—")</f>
+        <v>Vinnare</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B19" s="20" t="str">
-        <f aca="false">IFERROR(INDEX(Matcher!C:C,COUNTA(Matcher!A:A)-1-2+1),"—")</f>
-        <v>Slutade</v>
-      </c>
-      <c r="C19" s="20" t="str">
-        <f aca="false">IFERROR(INDEX(Matcher!J:J,COUNTA(Matcher!A:A)-1-2+1),"—")</f>
-        <v>Lag 1</v>
+      <c r="B19" s="20" t="n">
+        <f aca="false">IFERROR(INDEX(Matcher!D:D,COUNTA(Matcher!B:B)-1-2+1),"—")</f>
+        <v>0</v>
+      </c>
+      <c r="C19" s="20" t="n">
+        <f aca="false">IFERROR(INDEX(Matcher!K:K,COUNTA(Matcher!B:B)-1-2+1),"—")</f>
+        <v>0</v>
       </c>
       <c r="D19" s="20" t="str">
-        <f aca="false">IFERROR(INDEX(Matcher!K:K,COUNTA(Matcher!A:A)-1-2+1)&amp;" – "&amp;INDEX(Matcher!M:M,COUNTA(Matcher!A:A)-1-2+1),"—")</f>
-        <v>Poäng 1 – Poäng 2</v>
-      </c>
-      <c r="E19" s="20" t="str">
-        <f aca="false">IFERROR(INDEX(Matcher!L:L,COUNTA(Matcher!A:A)-1-2+1),"—")</f>
-        <v>Lag 2</v>
-      </c>
-      <c r="F19" s="20" t="str">
-        <f aca="false">IFERROR(INDEX(Matcher!N:N,COUNTA(Matcher!A:A)-1-2+1),"—")</f>
-        <v>Vinnare</v>
+        <f aca="false">IFERROR(INDEX(Matcher!M:M,COUNTA(Matcher!B:B)-1-2+1)&amp;" – "&amp;INDEX(Matcher!P:P,COUNTA(Matcher!B:B)-1-2+1),"—")</f>
+        <v> – </v>
+      </c>
+      <c r="E19" s="20" t="n">
+        <f aca="false">IFERROR(INDEX(Matcher!N:N,COUNTA(Matcher!B:B)-1-2+1),"—")</f>
+        <v>0</v>
+      </c>
+      <c r="F19" s="20" t="n">
+        <f aca="false">IFERROR(INDEX(Matcher!Q:Q,COUNTA(Matcher!B:B)-1-2+1),"—")</f>
+        <v>0</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B20" s="20" t="n">
-        <f aca="false">IFERROR(INDEX(Matcher!C:C,COUNTA(Matcher!A:A)-1-3+1),"—")</f>
-        <v>0</v>
-      </c>
-      <c r="C20" s="20" t="n">
-        <f aca="false">IFERROR(INDEX(Matcher!J:J,COUNTA(Matcher!A:A)-1-3+1),"—")</f>
-        <v>0</v>
+      <c r="B20" s="20" t="str">
+        <f aca="false">IFERROR(INDEX(Matcher!D:D,COUNTA(Matcher!B:B)-1-3+1),"—")</f>
+        <v>—</v>
+      </c>
+      <c r="C20" s="20" t="str">
+        <f aca="false">IFERROR(INDEX(Matcher!K:K,COUNTA(Matcher!B:B)-1-3+1),"—")</f>
+        <v>—</v>
       </c>
       <c r="D20" s="20" t="str">
-        <f aca="false">IFERROR(INDEX(Matcher!K:K,COUNTA(Matcher!A:A)-1-3+1)&amp;" – "&amp;INDEX(Matcher!M:M,COUNTA(Matcher!A:A)-1-3+1),"—")</f>
-        <v> – </v>
-      </c>
-      <c r="E20" s="20" t="n">
-        <f aca="false">IFERROR(INDEX(Matcher!L:L,COUNTA(Matcher!A:A)-1-3+1),"—")</f>
-        <v>0</v>
-      </c>
-      <c r="F20" s="20" t="n">
-        <f aca="false">IFERROR(INDEX(Matcher!N:N,COUNTA(Matcher!A:A)-1-3+1),"—")</f>
-        <v>0</v>
+        <f aca="false">IFERROR(INDEX(Matcher!M:M,COUNTA(Matcher!B:B)-1-3+1)&amp;" – "&amp;INDEX(Matcher!P:P,COUNTA(Matcher!B:B)-1-3+1),"—")</f>
+        <v>—</v>
+      </c>
+      <c r="E20" s="20" t="str">
+        <f aca="false">IFERROR(INDEX(Matcher!N:N,COUNTA(Matcher!B:B)-1-3+1),"—")</f>
+        <v>—</v>
+      </c>
+      <c r="F20" s="20" t="str">
+        <f aca="false">IFERROR(INDEX(Matcher!Q:Q,COUNTA(Matcher!B:B)-1-3+1),"—")</f>
+        <v>—</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B21" s="20" t="str">
-        <f aca="false">IFERROR(INDEX(Matcher!C:C,COUNTA(Matcher!A:A)-1-4+1),"—")</f>
+        <f aca="false">IFERROR(INDEX(Matcher!D:D,COUNTA(Matcher!B:B)-1-4+1),"—")</f>
         <v>—</v>
       </c>
       <c r="C21" s="20" t="str">
-        <f aca="false">IFERROR(INDEX(Matcher!J:J,COUNTA(Matcher!A:A)-1-4+1),"—")</f>
+        <f aca="false">IFERROR(INDEX(Matcher!K:K,COUNTA(Matcher!B:B)-1-4+1),"—")</f>
         <v>—</v>
       </c>
       <c r="D21" s="20" t="str">
-        <f aca="false">IFERROR(INDEX(Matcher!K:K,COUNTA(Matcher!A:A)-1-4+1)&amp;" – "&amp;INDEX(Matcher!M:M,COUNTA(Matcher!A:A)-1-4+1),"—")</f>
+        <f aca="false">IFERROR(INDEX(Matcher!M:M,COUNTA(Matcher!B:B)-1-4+1)&amp;" – "&amp;INDEX(Matcher!P:P,COUNTA(Matcher!B:B)-1-4+1),"—")</f>
         <v>—</v>
       </c>
       <c r="E21" s="20" t="str">
-        <f aca="false">IFERROR(INDEX(Matcher!L:L,COUNTA(Matcher!A:A)-1-4+1),"—")</f>
+        <f aca="false">IFERROR(INDEX(Matcher!N:N,COUNTA(Matcher!B:B)-1-4+1),"—")</f>
         <v>—</v>
       </c>
       <c r="F21" s="20" t="str">
-        <f aca="false">IFERROR(INDEX(Matcher!N:N,COUNTA(Matcher!A:A)-1-4+1),"—")</f>
+        <f aca="false">IFERROR(INDEX(Matcher!Q:Q,COUNTA(Matcher!B:B)-1-4+1),"—")</f>
         <v>—</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="21" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="C24" s="21"/>
       <c r="D24" s="21"/>

</xml_diff>

<commit_message>
Template: add Lagsättningar and Spelare tabs as physical sheets
</commit_message>
<xml_diff>
--- a/Boule-matcher-mall.xlsx
+++ b/Boule-matcher-mall.xlsx
@@ -11,7 +11,9 @@
     <sheet name="Instruktioner" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Apps Script-kod" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Matcher" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Sammanfattning" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Lagsättningar" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Spelare" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Sammanfattning" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="79">
   <si>
     <t xml:space="preserve">Boule Score Tracker</t>
   </si>
@@ -348,6 +350,42 @@
     <t xml:space="preserve">Raden ovan är bara ett exempel — du kan radera den. När Apps Script-webhooken är igång kommer varje avslutad match i appen skapa en ny rad här.</t>
   </si>
   <si>
+    <t xml:space="preserve">Lag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lagnamn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spelare</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anna</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Erik</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Johan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En rad per spelare och match. Fylls på automatiskt av webhooken. Du kan ta bort exempelraderna ovan.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Matcher</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vinster</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Senast sedd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Webhooken underhåller denna flik automatiskt. Varje spelare får en rad med totalt antal matcher, vinster och när de senast spelade.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Sammanfattning</t>
   </si>
   <si>
@@ -370,9 +408,6 @@
   </si>
   <si>
     <t xml:space="preserve">Per lag</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lag</t>
   </si>
   <si>
     <t xml:space="preserve">Segrar</t>
@@ -619,6 +654,10 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -653,10 +692,6 @@
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1245,6 +1280,234 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="B7" s="12"/>
+      <c r="C7" s="12"/>
+      <c r="D7" s="12"/>
+      <c r="E7" s="12"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A7:E7"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="24"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="B2" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="B3" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="B4" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="B5" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="B7" s="12"/>
+      <c r="C7" s="12"/>
+      <c r="D7" s="12"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A7:D7"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="B1:F24"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -1256,253 +1519,253 @@
     <row r="1" customFormat="false" ht="9.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="2" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="2" t="s">
-        <v>53</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="9.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B5" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="C5" s="13" t="n">
+      <c r="B5" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="C5" s="14" t="n">
         <f aca="false">COUNTA(Matcher!Q:Q)-1</f>
         <v>1</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="C6" s="13" t="n">
+      <c r="B6" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="C6" s="14" t="n">
         <f aca="false">COUNTIF(Matcher!Q:Q,"Tjejerna")</f>
         <v>1</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="C7" s="13" t="n">
+      <c r="B7" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="C7" s="14" t="n">
         <f aca="false">COUNTIF(Matcher!Q:Q,"Killarna")</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="12" t="s">
-        <v>57</v>
-      </c>
-      <c r="C8" s="14" t="n">
+      <c r="B8" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="C8" s="15" t="n">
         <f aca="false">IFERROR(AVERAGE(Matcher!R2:R1000),0)</f>
         <v>11</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="C9" s="13" t="n">
-        <f aca="false">IFERROR(COUNTA(spelare!a:a)-1,0)</f>
-        <v>0</v>
+      <c r="B9" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="C9" s="14" t="n">
+        <f aca="false">IFERROR(COUNTA(Spelare!A:A)-1,0)</f>
+        <v>5</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="15" t="s">
-        <v>59</v>
+      <c r="B10" s="16" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="16" t="s">
-        <v>60</v>
-      </c>
-      <c r="C11" s="16" t="s">
-        <v>61</v>
-      </c>
-      <c r="D11" s="16" t="s">
-        <v>62</v>
-      </c>
-      <c r="E11" s="16" t="s">
-        <v>63</v>
+      <c r="B11" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="C11" s="17" t="s">
+        <v>72</v>
+      </c>
+      <c r="D11" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="E11" s="17" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B12" s="17" t="s">
+      <c r="B12" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="C12" s="18" t="n">
+      <c r="C12" s="19" t="n">
         <f aca="false">COUNTIF(Matcher!Q:Q,B12)</f>
         <v>1</v>
       </c>
-      <c r="D12" s="18" t="n">
+      <c r="D12" s="19" t="n">
         <f aca="false">SUMIF(Matcher!K:K,B12,Matcher!M:M)+SUMIF(Matcher!N:N,B12,Matcher!P:P)</f>
         <v>13</v>
       </c>
-      <c r="E12" s="19" t="str">
+      <c r="E12" s="20" t="str">
         <f aca="false">IFERROR(maxifs(Matcher!D:D,Matcher!Q:Q,B12),"—")</f>
         <v>—</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B13" s="17" t="s">
+      <c r="B13" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="C13" s="18" t="n">
+      <c r="C13" s="19" t="n">
         <f aca="false">COUNTIF(Matcher!Q:Q,B13)</f>
         <v>0</v>
       </c>
-      <c r="D13" s="18" t="n">
+      <c r="D13" s="19" t="n">
         <f aca="false">SUMIF(Matcher!K:K,B13,Matcher!M:M)+SUMIF(Matcher!N:N,B13,Matcher!P:P)</f>
         <v>9</v>
       </c>
-      <c r="E13" s="19" t="str">
+      <c r="E13" s="20" t="str">
         <f aca="false">IFERROR(maxifs(Matcher!D:D,Matcher!Q:Q,B13),"—")</f>
         <v>—</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="15" t="s">
-        <v>64</v>
+      <c r="B15" s="16" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B16" s="16" t="s">
-        <v>65</v>
-      </c>
-      <c r="C16" s="16" t="s">
+      <c r="B16" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="C16" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="D16" s="16" t="s">
-        <v>66</v>
-      </c>
-      <c r="E16" s="16" t="s">
+      <c r="D16" s="17" t="s">
+        <v>77</v>
+      </c>
+      <c r="E16" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="F16" s="16" t="s">
+      <c r="F16" s="17" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B17" s="20" t="str">
+      <c r="B17" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Matcher!D:D,COUNTA(Matcher!B:B)-1-0+1),"—")</f>
         <v>2026-04-18T20:15:28.000Z</v>
       </c>
-      <c r="C17" s="20" t="str">
+      <c r="C17" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Matcher!K:K,COUNTA(Matcher!B:B)-1-0+1),"—")</f>
         <v>Tjejerna</v>
       </c>
-      <c r="D17" s="20" t="str">
+      <c r="D17" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Matcher!M:M,COUNTA(Matcher!B:B)-1-0+1)&amp;" – "&amp;INDEX(Matcher!P:P,COUNTA(Matcher!B:B)-1-0+1),"—")</f>
         <v>13 – 9</v>
       </c>
-      <c r="E17" s="20" t="str">
+      <c r="E17" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Matcher!N:N,COUNTA(Matcher!B:B)-1-0+1),"—")</f>
         <v>Killarna</v>
       </c>
-      <c r="F17" s="20" t="str">
+      <c r="F17" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Matcher!Q:Q,COUNTA(Matcher!B:B)-1-0+1),"—")</f>
         <v>Tjejerna</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="20" t="str">
+      <c r="B18" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Matcher!D:D,COUNTA(Matcher!B:B)-1-1+1),"—")</f>
         <v>Slutade</v>
       </c>
-      <c r="C18" s="20" t="str">
+      <c r="C18" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Matcher!K:K,COUNTA(Matcher!B:B)-1-1+1),"—")</f>
         <v>Lag 1</v>
       </c>
-      <c r="D18" s="20" t="str">
+      <c r="D18" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Matcher!M:M,COUNTA(Matcher!B:B)-1-1+1)&amp;" – "&amp;INDEX(Matcher!P:P,COUNTA(Matcher!B:B)-1-1+1),"—")</f>
         <v>Poäng 1 – Poäng 2</v>
       </c>
-      <c r="E18" s="20" t="str">
+      <c r="E18" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Matcher!N:N,COUNTA(Matcher!B:B)-1-1+1),"—")</f>
         <v>Lag 2</v>
       </c>
-      <c r="F18" s="20" t="str">
+      <c r="F18" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Matcher!Q:Q,COUNTA(Matcher!B:B)-1-1+1),"—")</f>
         <v>Vinnare</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B19" s="20" t="n">
+      <c r="B19" s="21" t="n">
         <f aca="false">IFERROR(INDEX(Matcher!D:D,COUNTA(Matcher!B:B)-1-2+1),"—")</f>
         <v>0</v>
       </c>
-      <c r="C19" s="20" t="n">
+      <c r="C19" s="21" t="n">
         <f aca="false">IFERROR(INDEX(Matcher!K:K,COUNTA(Matcher!B:B)-1-2+1),"—")</f>
         <v>0</v>
       </c>
-      <c r="D19" s="20" t="str">
+      <c r="D19" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Matcher!M:M,COUNTA(Matcher!B:B)-1-2+1)&amp;" – "&amp;INDEX(Matcher!P:P,COUNTA(Matcher!B:B)-1-2+1),"—")</f>
         <v> – </v>
       </c>
-      <c r="E19" s="20" t="n">
+      <c r="E19" s="21" t="n">
         <f aca="false">IFERROR(INDEX(Matcher!N:N,COUNTA(Matcher!B:B)-1-2+1),"—")</f>
         <v>0</v>
       </c>
-      <c r="F19" s="20" t="n">
+      <c r="F19" s="21" t="n">
         <f aca="false">IFERROR(INDEX(Matcher!Q:Q,COUNTA(Matcher!B:B)-1-2+1),"—")</f>
         <v>0</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B20" s="20" t="str">
+      <c r="B20" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Matcher!D:D,COUNTA(Matcher!B:B)-1-3+1),"—")</f>
         <v>—</v>
       </c>
-      <c r="C20" s="20" t="str">
+      <c r="C20" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Matcher!K:K,COUNTA(Matcher!B:B)-1-3+1),"—")</f>
         <v>—</v>
       </c>
-      <c r="D20" s="20" t="str">
+      <c r="D20" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Matcher!M:M,COUNTA(Matcher!B:B)-1-3+1)&amp;" – "&amp;INDEX(Matcher!P:P,COUNTA(Matcher!B:B)-1-3+1),"—")</f>
         <v>—</v>
       </c>
-      <c r="E20" s="20" t="str">
+      <c r="E20" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Matcher!N:N,COUNTA(Matcher!B:B)-1-3+1),"—")</f>
         <v>—</v>
       </c>
-      <c r="F20" s="20" t="str">
+      <c r="F20" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Matcher!Q:Q,COUNTA(Matcher!B:B)-1-3+1),"—")</f>
         <v>—</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="20" t="str">
+      <c r="B21" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Matcher!D:D,COUNTA(Matcher!B:B)-1-4+1),"—")</f>
         <v>—</v>
       </c>
-      <c r="C21" s="20" t="str">
+      <c r="C21" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Matcher!K:K,COUNTA(Matcher!B:B)-1-4+1),"—")</f>
         <v>—</v>
       </c>
-      <c r="D21" s="20" t="str">
+      <c r="D21" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Matcher!M:M,COUNTA(Matcher!B:B)-1-4+1)&amp;" – "&amp;INDEX(Matcher!P:P,COUNTA(Matcher!B:B)-1-4+1),"—")</f>
         <v>—</v>
       </c>
-      <c r="E21" s="20" t="str">
+      <c r="E21" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Matcher!N:N,COUNTA(Matcher!B:B)-1-4+1),"—")</f>
         <v>—</v>
       </c>
-      <c r="F21" s="20" t="str">
+      <c r="F21" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Matcher!Q:Q,COUNTA(Matcher!B:B)-1-4+1),"—")</f>
         <v>—</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="C24" s="21"/>
-      <c r="D24" s="21"/>
-      <c r="E24" s="21"/>
-      <c r="F24" s="21"/>
+      <c r="B24" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="C24" s="12"/>
+      <c r="D24" s="12"/>
+      <c r="E24" s="12"/>
+      <c r="F24" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>